<commit_message>
index viaje a italia
</commit_message>
<xml_diff>
--- a/viaje/GASTOS ROMA.xlsx
+++ b/viaje/GASTOS ROMA.xlsx
@@ -7,8 +7,8 @@
     <workbookView xWindow="480" yWindow="36" windowWidth="22116" windowHeight="10872"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="GASTOS TOTALES DE ITALIA" sheetId="1" r:id="rId1"/>
+    <sheet name="GASTOS EN ITALIA" sheetId="2" r:id="rId2"/>
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="77">
   <si>
     <t>IBERIA</t>
   </si>
@@ -208,6 +208,84 @@
   </si>
   <si>
     <t>equipaje de mano (56,40,25) &lt;10Kg + equipaje &lt;23kg (selección asiento desde 24h)</t>
+  </si>
+  <si>
+    <t>GASTOS EN ITALIA</t>
+  </si>
+  <si>
+    <t>LUGAR</t>
+  </si>
+  <si>
+    <t>McDonalds helado</t>
+  </si>
+  <si>
+    <t>carrefour express</t>
+  </si>
+  <si>
+    <t>McDonalds patatas</t>
+  </si>
+  <si>
+    <t>comida aeropuerto Roma llegada: agua y pizza</t>
+  </si>
+  <si>
+    <t>pago llegada alojamiento Roma</t>
+  </si>
+  <si>
+    <t>metro Roma</t>
+  </si>
+  <si>
+    <t>Café en Florencia, 2 cafés</t>
+  </si>
+  <si>
+    <t>Supermercado Tigre</t>
+  </si>
+  <si>
+    <t>Transacción online día 13 del cambio..</t>
+  </si>
+  <si>
+    <t>Transacción 11 de diciembre no sé de qué</t>
+  </si>
+  <si>
+    <t>La bottega del café Siena Fruta en vaso</t>
+  </si>
+  <si>
+    <t>Supermercado Pam en Siena</t>
+  </si>
+  <si>
+    <t>Cena en Florencia Lántica Fraschetta</t>
+  </si>
+  <si>
+    <t>Ufizi postales</t>
+  </si>
+  <si>
+    <t>Edoardo Florencia helado</t>
+  </si>
+  <si>
+    <t>il Bargello Siena (espaguetis gruesos)</t>
+  </si>
+  <si>
+    <t>Helados en Roma</t>
+  </si>
+  <si>
+    <t>Pizza en mercado de Florencia</t>
+  </si>
+  <si>
+    <t>MULTA TRANVIA</t>
+  </si>
+  <si>
+    <t>LLEGADA TARDE A BARJAS</t>
+  </si>
+  <si>
+    <t>LOS DOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuchillo puntilla </t>
+  </si>
+  <si>
+    <t>pasta en bote 11 de junio</t>
+  </si>
+  <si>
+    <t>POR CABEZA</t>
   </si>
 </sst>
 </file>
@@ -219,7 +297,7 @@
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,6 +350,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -319,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -354,6 +439,7 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -655,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
@@ -993,29 +1079,49 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="21">
-        <f>SUM(B2:B18)</f>
-        <v>2007.24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E22" s="1">
+      <c r="A20" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="19">
+        <f>'GASTOS EN ITALIA'!B28</f>
+        <v>555.99</v>
+      </c>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="21">
+        <f>SUM(B2:B20)</f>
+        <v>2575.23</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21">
+        <f>B21/2</f>
+        <v>1287.615</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E23" s="1">
         <v>1839</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E24" s="1">
-        <f>E22*2</f>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E25" s="1">
+        <f>E23*2</f>
         <v>3678</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E25">
-        <f>E24-B20</f>
-        <v>1670.76</v>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E26">
+        <f>E25-B21</f>
+        <v>1102.77</v>
       </c>
     </row>
   </sheetData>
@@ -1027,9 +1133,234 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="39.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="5"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="5">
+        <v>2.5499999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="5">
+        <v>8.4499999999999993</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="5">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="5">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="22">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="5">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="5">
+        <v>6.95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="5">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="5">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="5">
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="5">
+        <v>12.19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="5">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="5">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="5">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="5">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="5">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="5">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="5"/>
+      <c r="B28" s="7">
+        <f>SUM(B2:B27)</f>
+        <v>555.99</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>